<commit_message>
One file for multicurrencies+
</commit_message>
<xml_diff>
--- a/inputs/Regions_countries_list.xlsx
+++ b/inputs/Regions_countries_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hrtelekom-my.sharepoint.com/personal/diego_deblock_t_ht_hr/Documents/Documents/Python/TT-Robopricing/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:20000001_{A28FD2E6-A31D-4B8B-AAFF-80AF378F6979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FD5AD19-C557-4B97-9806-F5AD97EAA37C}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:20000001_{A28FD2E6-A31D-4B8B-AAFF-80AF378F6979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECB20937-7C20-4850-BE1F-25F5B620A45F}"/>
   <bookViews>
-    <workbookView xWindow="5730" yWindow="2910" windowWidth="38700" windowHeight="15345" xr2:uid="{69DE24D8-959D-4BE0-AF31-341EA28F7D69}"/>
+    <workbookView xWindow="2160" yWindow="2160" windowWidth="17745" windowHeight="15465" activeTab="4" xr2:uid="{69DE24D8-959D-4BE0-AF31-341EA28F7D69}"/>
   </bookViews>
   <sheets>
     <sheet name="Regions" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">MappingTable!$A$1:$H$186</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -75,7 +76,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
-Type region  from Region sheet to get list of the countries!</t>
+Type region number  from Region sheet to get list of the countries!</t>
         </r>
       </text>
     </comment>
@@ -26081,6 +26082,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007113BAA1CEDDFC45BBB3E5AE2B53E5DC" ma:contentTypeVersion="0" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="45a76d64ae33887ad6306091372d873e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1b05d82d297216baf5b26c55225140df">
     <xsd:element name="properties">
@@ -26194,7 +26201,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -26203,13 +26210,22 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DABA9059-20BA-4E74-9CEF-48B872B3B8DC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E341464-ADDE-4AB7-8F54-65E658F8D3D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -26225,25 +26241,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05BAF265-B1CE-46B5-B635-099AD1D09506}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DABA9059-20BA-4E74-9CEF-48B872B3B8DC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>